<commit_message>
Fix vendor master data in Excel templates
- LLS電気株式会社 → LLS電気（個人事業主）
- トラストテクノス株式会社 → 株式会社トラストテクノス（法人）

Updated both 経営管理_テンプレート.xlsx and 年間サマリー_テンプレート.xlsx

https://claude.ai/code/session_01Q6cChDrZgyWiB9miRXTLrq
</commit_message>
<xml_diff>
--- a/excel-templates/年間サマリー_テンプレート.xlsx
+++ b/excel-templates/年間サマリー_テンプレート.xlsx
@@ -985,7 +985,7 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>LLS電気株式会社</t>
+          <t>LLS電気</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -1008,7 +1008,7 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>トラストテクノス株式会社</t>
+          <t>株式会社トラストテクノス</t>
         </is>
       </c>
       <c r="B6" s="3" t="n"/>

</xml_diff>